<commit_message>
docs(testing): preserve C-109 flag priority in cases
E06-S06 / SCRUM-50, follow-up to #339. Correct only TC_E06S06_01/_06 descriptions and regenerate matching dated/current payloads; both approvals still refuse until explicit resolution.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 221026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 221026.xlsx
@@ -10964,7 +10964,7 @@
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm the buffer edit saves and affected bookings remain present with the `buffer_conflict` flag.
+          <t>1. Confirm the buffer edit saves and both bookings remain present; Pending Product Expo has `buffer_conflict` true while Confirmed Charity Run remains unflagged.
 2. Open Product Expo's Pending request and attempt approval.</t>
         </is>
       </c>
@@ -10975,7 +10975,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>Approval is refused after checking current buffers. The Confirmed booking and Pending request are retained, their conflict remains flagged, and neither is silently released.</t>
+          <t>Approval of Product Expo is refused after checking current buffers. Confirmed Charity Run and Pending Product Expo are both retained; Charity Run remains unflagged and Product Expo carries `buffer_conflict` true.</t>
         </is>
       </c>
     </row>
@@ -11219,7 +11219,7 @@
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm the buffer edit saves, both Pending rows remain, and both show `buffer_conflict`.
+          <t>1. Confirm the buffer edit saves and both Pending rows remain; earlier Charity Run is unflagged and later Alumni Dinner has `buffer_conflict` true under the existing equal-status ordering.
 2. Attempt approval of each request while the buffered conflict remains.
 3. Resolve the conflict using one of these paths: (primary) Venue Staff reject one conflicting Pending request with a reason; (alternative) an authorized Coordinator withdraws/replans one request to a nonconflicting period and resubmits it as needed.
 4. Approve the remaining now-free Pending request. For the alternative path, also approve the replanned request only if it is Pending and conflict-free.</t>
@@ -11232,7 +11232,7 @@
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>Both approvals are refused while the conflict remains, and there is no automatic winner. The primary resolution is for Venue Staff to reject one conflicting Pending request with a reason; that row becomes terminal Rejected, and the remaining still-Pending request can then be approved. Alternatively, an authorized Coordinator may withdraw/replan one request to a nonconflicting period; the remaining now-free Pending request and any valid replanned Pending request can then be approved. A Rejected row is never approved.</t>
+          <t>Both approvals are refused while the conflict remains, and there is no automatic winner. Equal-status ordering leaves earlier Charity Run unflagged and sets `buffer_conflict` true on later Alumni Dinner. The primary resolution is for Venue Staff to reject one conflicting Pending request with a reason; that row becomes terminal Rejected, and the remaining still-Pending request can then be approved. Alternatively, an authorized Coordinator may withdraw/replan one request to a nonconflicting period; the remaining now-free Pending request and any valid replanned Pending request can then be approved. A Rejected row is never approved.</t>
         </is>
       </c>
     </row>

</xml_diff>